<commit_message>
feat: replace DashboardUsers with ConfigReportUsers/ConfigDashboards/DashboardAccess
- New 3-table auth schema: ConfigReportUsers, ConfigDashboards, DashboardAccess
- Migration script: sql/create_new_auth_tables.sql
- All auth endpoints (login, signup, forgot/reset password, admin approve/reject/remove)
  now use new tables; zero DashboardUsers references remain
- SLA_DASHBOARD_ID constant matches actual DB row (DashboardID=0)
- Fixed IsActive BIT boolean comparison (mssql returns bool not int)
- Admin users excluded from User Management list (self-managed)
- Added DELETE /api/admin/users/:id endpoint (permanent remove)
- Added Remove button to User Management (pending + all users tables)
- Renamed Company column to Staff Full Name, then removed it per request
- Fixed request() in api.js to accept options (enables DELETE method)
- Approve/Reject status now persists correctly across logout/login
</commit_message>
<xml_diff>
--- a/docs/SLA_Logic_Audit_2026-06-12.xlsx
+++ b/docs/SLA_Logic_Audit_2026-06-12.xlsx
@@ -8,25 +8,40 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mortgageezy-my.sharepoint.com/personal/ntruong_mezy_com_au/Documents/Project_VibeCoding/SLA Dashboard/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="90" documentId="11_5D8F141A1147CD0E743206136036A5F500A68C6A" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{310C260E-2889-40A9-8186-5B0F99F3877B}"/>
+  <xr:revisionPtr revIDLastSave="135" documentId="11_5D8F141A1147CD0E743206136036A5F500A68C6A" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3B6DD74B-5067-47E0-92CF-536774943CDC}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="33315" yWindow="2010" windowWidth="18660" windowHeight="12525" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SLA Logic Audit" sheetId="1" r:id="rId1"/>
     <sheet name="Summary" sheetId="2" r:id="rId2"/>
     <sheet name="Logins" sheetId="3" r:id="rId3"/>
     <sheet name="Cloudflare" sheetId="4" r:id="rId4"/>
+    <sheet name="Vercel" sheetId="5" r:id="rId5"/>
+    <sheet name="GoDaddy" sheetId="6" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'SLA Logic Audit'!$A$1:$F$15</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="155">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="167">
   <si>
     <t>Figure / Area</t>
   </si>
@@ -591,6 +606,9 @@
     <t xml:space="preserve">Token </t>
   </si>
   <si>
+    <t>Nuy...30!</t>
+  </si>
+  <si>
     <t xml:space="preserve">Password </t>
   </si>
   <si>
@@ -646,13 +664,46 @@
   </si>
   <si>
     <t>rob.ns.cloudflare.com</t>
+  </si>
+  <si>
+    <t>sla-dashboard - Overview – Vercel</t>
+  </si>
+  <si>
+    <t>https://vercel.com/mezyproject2026/sla-dashboard/settings/domains?domainconnect-domain=sla.mezy.com.au</t>
+  </si>
+  <si>
+    <t>GoDdady</t>
+  </si>
+  <si>
+    <t>ntruong email</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Railway </t>
+  </si>
+  <si>
+    <t>Ngrok</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ngrok Link </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deployement </t>
+  </si>
+  <si>
+    <t>sla-dashboard – Deployments – Vercel</t>
+  </si>
+  <si>
+    <t>SLA Performance Dashboard — Mortgage Ezy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Try open this link on Monday </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -710,13 +761,36 @@
       <family val="2"/>
     </font>
     <font>
+      <u/>
+      <sz val="12"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="12"/>
       <color rgb="FF313131"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <u/>
+      <sz val="12"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -744,6 +818,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -824,10 +904,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -870,7 +951,6 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -898,9 +978,16 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="2" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -921,15 +1008,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>419100</xdr:colOff>
-      <xdr:row>9</xdr:row>
-      <xdr:rowOff>133350</xdr:rowOff>
+      <xdr:colOff>1096433</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>133349</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>94390</xdr:colOff>
-      <xdr:row>40</xdr:row>
-      <xdr:rowOff>79659</xdr:rowOff>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>83806</xdr:colOff>
+      <xdr:row>45</xdr:row>
+      <xdr:rowOff>79658</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -952,8 +1039,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="10410825" y="1990725"/>
-          <a:ext cx="6876190" cy="6200000"/>
+          <a:off x="8906933" y="3064932"/>
+          <a:ext cx="6871956" cy="6232809"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1047,6 +1134,99 @@
         <a:xfrm>
           <a:off x="0" y="8267700"/>
           <a:ext cx="4980952" cy="4352381"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>123825</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>180975</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>149254</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>57150</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3362CF4A-8684-10BD-AFF7-12556FA1AB55}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="123825" y="381000"/>
+          <a:ext cx="4826029" cy="4276725"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>647700</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>47625</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>30</xdr:col>
+      <xdr:colOff>531421</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>66398</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{80F547A8-EE49-5661-7D78-B7747AA44A1E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6819900" y="1247775"/>
+          <a:ext cx="15828571" cy="2219048"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1380,7 +1560,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr filterMode="1"/>
+  <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:G15"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1415,7 +1595,7 @@
       </c>
       <c r="G1" s="16"/>
     </row>
-    <row r="2" spans="1:7" ht="127.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" ht="127.5" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
@@ -1436,7 +1616,7 @@
       </c>
       <c r="G2" s="15"/>
     </row>
-    <row r="3" spans="1:7" ht="76.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" ht="76.5" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -1457,7 +1637,7 @@
       </c>
       <c r="G3" s="15"/>
     </row>
-    <row r="4" spans="1:7" ht="140.25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" ht="140.25" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>17</v>
       </c>
@@ -1478,7 +1658,7 @@
       </c>
       <c r="G4" s="15"/>
     </row>
-    <row r="5" spans="1:7" ht="114.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" ht="114.75" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>22</v>
       </c>
@@ -1520,7 +1700,7 @@
       </c>
       <c r="G6" s="15"/>
     </row>
-    <row r="7" spans="1:7" ht="127.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" ht="127.5" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>32</v>
       </c>
@@ -1541,7 +1721,7 @@
       </c>
       <c r="G7" s="15"/>
     </row>
-    <row r="8" spans="1:7" ht="140.25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" ht="140.25" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>37</v>
       </c>
@@ -1562,7 +1742,7 @@
       </c>
       <c r="G8" s="15"/>
     </row>
-    <row r="9" spans="1:7" ht="76.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" ht="76.5" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>42</v>
       </c>
@@ -1583,7 +1763,7 @@
       </c>
       <c r="G9" s="15"/>
     </row>
-    <row r="10" spans="1:7" ht="76.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" ht="76.5" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>47</v>
       </c>
@@ -1604,7 +1784,7 @@
       </c>
       <c r="G10" s="15"/>
     </row>
-    <row r="11" spans="1:7" ht="267.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" ht="267.75" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>52</v>
       </c>
@@ -1625,7 +1805,7 @@
       </c>
       <c r="G11" s="15"/>
     </row>
-    <row r="12" spans="1:7" ht="178.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" ht="178.5" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>57</v>
       </c>
@@ -1646,7 +1826,7 @@
       </c>
       <c r="G12" s="15"/>
     </row>
-    <row r="13" spans="1:7" ht="229.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" ht="229.5" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>62</v>
       </c>
@@ -1667,7 +1847,7 @@
       </c>
       <c r="G13" s="15"/>
     </row>
-    <row r="14" spans="1:7" ht="153" hidden="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" ht="153" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>67</v>
       </c>
@@ -1688,7 +1868,7 @@
       </c>
       <c r="G14" s="15"/>
     </row>
-    <row r="15" spans="1:7" ht="204" hidden="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" ht="204" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>72</v>
       </c>
@@ -1710,13 +1890,7 @@
       <c r="G15" s="15"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F15" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <filterColumn colId="0">
-      <filters>
-        <filter val="Overall KPI — Total Active Tasks"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:F15" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
     <ignoredError sqref="A1:F15" numberStoredAsText="1"/>
@@ -1726,6 +1900,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <sheetPr codeName="Sheet2"/>
   <dimension ref="A1:C25"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
@@ -1949,10 +2124,11 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FF817616-9591-4502-ADA5-31304F08E7DC}">
-  <dimension ref="A3:I17"/>
+  <sheetPr codeName="Sheet3"/>
+  <dimension ref="A3:I25"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="30.375" customWidth="1"/>
+    <col min="1" max="1" width="41.75" customWidth="1"/>
     <col min="2" max="2" width="14.75" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="16.75" bestFit="1" customWidth="1"/>
     <col min="4" max="6" width="14.625" bestFit="1" customWidth="1"/>
@@ -1964,231 +2140,363 @@
       <c r="A3" s="17" t="s">
         <v>113</v>
       </c>
-      <c r="B3" s="18"/>
-      <c r="C3" s="18"/>
-      <c r="D3" s="18"/>
-      <c r="E3" s="18"/>
-      <c r="F3" s="18"/>
-      <c r="G3" s="18"/>
-      <c r="H3" s="18"/>
-      <c r="I3" s="18"/>
+      <c r="B3" s="10"/>
+      <c r="C3" s="10"/>
+      <c r="D3" s="10"/>
+      <c r="E3" s="10"/>
+      <c r="F3" s="10"/>
+      <c r="G3" s="10"/>
+      <c r="H3" s="10"/>
+      <c r="I3" s="10"/>
     </row>
     <row r="4" spans="1:9" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="19" t="s">
+      <c r="A4" s="18" t="s">
         <v>114</v>
       </c>
-      <c r="B4" s="20" t="s">
+      <c r="B4" s="19" t="s">
         <v>115</v>
       </c>
-      <c r="C4" s="20" t="s">
+      <c r="C4" s="19" t="s">
         <v>116</v>
       </c>
-      <c r="D4" s="20" t="s">
+      <c r="D4" s="19" t="s">
         <v>117</v>
       </c>
-      <c r="E4" s="24" t="s">
+      <c r="E4" s="23" t="s">
         <v>133</v>
       </c>
-      <c r="F4" s="24" t="s">
+      <c r="F4" s="23" t="s">
         <v>134</v>
       </c>
-      <c r="G4" s="24" t="s">
+      <c r="G4" s="23" t="s">
+        <v>137</v>
+      </c>
+      <c r="H4" s="23" t="s">
+        <v>135</v>
+      </c>
+      <c r="I4" s="23"/>
+    </row>
+    <row r="5" spans="1:9" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="20" t="s">
+        <v>118</v>
+      </c>
+      <c r="B5" s="21" t="s">
+        <v>119</v>
+      </c>
+      <c r="C5" s="22" t="s">
+        <v>120</v>
+      </c>
+      <c r="D5" s="22" t="s">
+        <v>121</v>
+      </c>
+      <c r="E5" s="24"/>
+      <c r="F5" s="24"/>
+      <c r="G5" s="24"/>
+      <c r="H5" s="24"/>
+      <c r="I5" s="24"/>
+    </row>
+    <row r="6" spans="1:9" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="20" t="s">
+        <v>122</v>
+      </c>
+      <c r="B6" s="21" t="s">
+        <v>123</v>
+      </c>
+      <c r="C6" s="22" t="s">
+        <v>124</v>
+      </c>
+      <c r="D6" s="22" t="s">
+        <v>125</v>
+      </c>
+      <c r="E6" s="24"/>
+      <c r="F6" s="24"/>
+      <c r="G6" s="24"/>
+      <c r="H6" s="24"/>
+      <c r="I6" s="24"/>
+    </row>
+    <row r="7" spans="1:9" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="20" t="s">
+        <v>126</v>
+      </c>
+      <c r="B7" s="21" t="s">
+        <v>127</v>
+      </c>
+      <c r="C7" s="22" t="s">
+        <v>128</v>
+      </c>
+      <c r="D7" s="22" t="s">
+        <v>125</v>
+      </c>
+      <c r="E7" s="24"/>
+      <c r="F7" s="24"/>
+      <c r="G7" s="24"/>
+      <c r="H7" s="24"/>
+      <c r="I7" s="24"/>
+    </row>
+    <row r="8" spans="1:9" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="20" t="s">
+        <v>129</v>
+      </c>
+      <c r="B8" s="22" t="s">
+        <v>130</v>
+      </c>
+      <c r="C8" s="22" t="s">
+        <v>131</v>
+      </c>
+      <c r="D8" s="22" t="s">
+        <v>132</v>
+      </c>
+      <c r="E8" s="24"/>
+      <c r="F8" s="24"/>
+      <c r="G8" s="24" t="s">
+        <v>138</v>
+      </c>
+      <c r="H8" s="24"/>
+      <c r="I8" s="24"/>
+    </row>
+    <row r="9" spans="1:9" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="20" t="s">
+        <v>139</v>
+      </c>
+      <c r="B9" s="22"/>
+      <c r="C9" s="22"/>
+      <c r="D9" s="22"/>
+      <c r="E9" s="24"/>
+      <c r="F9" s="24" t="s">
+        <v>140</v>
+      </c>
+      <c r="G9" s="24" t="s">
+        <v>140</v>
+      </c>
+      <c r="H9" s="24"/>
+      <c r="I9" s="24"/>
+    </row>
+    <row r="10" spans="1:9" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="20" t="s">
+        <v>141</v>
+      </c>
+      <c r="B10" s="22"/>
+      <c r="C10" s="22"/>
+      <c r="D10" s="22"/>
+      <c r="E10" s="24"/>
+      <c r="F10" s="24" t="s">
+        <v>140</v>
+      </c>
+      <c r="G10" s="24" t="s">
+        <v>140</v>
+      </c>
+      <c r="H10" s="24"/>
+      <c r="I10" s="24"/>
+    </row>
+    <row r="11" spans="1:9" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="20" t="s">
+        <v>158</v>
+      </c>
+      <c r="B11" s="22"/>
+      <c r="C11" s="22"/>
+      <c r="D11" s="22"/>
+      <c r="E11" s="24"/>
+      <c r="F11" s="24" t="s">
+        <v>159</v>
+      </c>
+      <c r="G11" s="24" t="s">
         <v>136</v>
       </c>
-      <c r="H4" s="24" t="s">
-        <v>135</v>
-      </c>
-      <c r="I4" s="24"/>
-    </row>
-    <row r="5" spans="1:9" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="21" t="s">
-        <v>118</v>
-      </c>
-      <c r="B5" s="22" t="s">
+      <c r="H11" s="24"/>
+      <c r="I11" s="24"/>
+    </row>
+    <row r="12" spans="1:9" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="20" t="s">
+        <v>160</v>
+      </c>
+      <c r="B12" s="22"/>
+      <c r="C12" s="22"/>
+      <c r="D12" s="22"/>
+      <c r="E12" s="24"/>
+      <c r="F12" s="24" t="s">
+        <v>140</v>
+      </c>
+      <c r="G12" s="24" t="s">
+        <v>140</v>
+      </c>
+      <c r="H12" s="24"/>
+      <c r="I12" s="24"/>
+    </row>
+    <row r="13" spans="1:9" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="20" t="s">
+        <v>161</v>
+      </c>
+      <c r="B13" s="22"/>
+      <c r="C13" s="22"/>
+      <c r="D13" s="22"/>
+      <c r="E13" s="29" t="s">
+        <v>162</v>
+      </c>
+      <c r="F13" s="24" t="s">
+        <v>140</v>
+      </c>
+      <c r="G13" s="24" t="s">
+        <v>140</v>
+      </c>
+      <c r="H13" s="24"/>
+      <c r="I13" s="24"/>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A14" s="28"/>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A15" s="28"/>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A16" s="28"/>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" s="28"/>
+    </row>
+    <row r="18" spans="1:3" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="26" t="s">
+        <v>142</v>
+      </c>
+      <c r="B18" s="21" t="s">
+        <v>143</v>
+      </c>
+      <c r="C18" s="25" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="20" t="s">
+        <v>145</v>
+      </c>
+      <c r="B19" s="22" t="s">
+        <v>146</v>
+      </c>
+      <c r="C19" s="22" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="20" t="s">
+        <v>148</v>
+      </c>
+      <c r="B20" s="22" t="s">
+        <v>149</v>
+      </c>
+      <c r="C20" s="22" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="20" t="s">
         <v>119</v>
       </c>
-      <c r="C5" s="23" t="s">
-        <v>120</v>
-      </c>
-      <c r="D5" s="23" t="s">
-        <v>121</v>
-      </c>
-      <c r="E5" s="25"/>
-      <c r="F5" s="25"/>
-      <c r="G5" s="25"/>
-      <c r="H5" s="25"/>
-      <c r="I5" s="25"/>
-    </row>
-    <row r="6" spans="1:9" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="21" t="s">
-        <v>122</v>
-      </c>
-      <c r="B6" s="22" t="s">
-        <v>123</v>
-      </c>
-      <c r="C6" s="23" t="s">
-        <v>124</v>
-      </c>
-      <c r="D6" s="23" t="s">
-        <v>125</v>
-      </c>
-      <c r="E6" s="25"/>
-      <c r="F6" s="25"/>
-      <c r="G6" s="25"/>
-      <c r="H6" s="25"/>
-      <c r="I6" s="25"/>
-    </row>
-    <row r="7" spans="1:9" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="21" t="s">
-        <v>126</v>
-      </c>
-      <c r="B7" s="22" t="s">
-        <v>127</v>
-      </c>
-      <c r="C7" s="23" t="s">
-        <v>128</v>
-      </c>
-      <c r="D7" s="23" t="s">
-        <v>125</v>
-      </c>
-      <c r="E7" s="25"/>
-      <c r="F7" s="25"/>
-      <c r="G7" s="25"/>
-      <c r="H7" s="25"/>
-      <c r="I7" s="25"/>
-    </row>
-    <row r="8" spans="1:9" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="21" t="s">
-        <v>129</v>
-      </c>
-      <c r="B8" s="23" t="s">
-        <v>130</v>
-      </c>
-      <c r="C8" s="23" t="s">
-        <v>131</v>
-      </c>
-      <c r="D8" s="23" t="s">
-        <v>132</v>
-      </c>
-      <c r="E8" s="25"/>
-      <c r="F8" s="25"/>
-      <c r="G8" s="25" t="s">
-        <v>137</v>
-      </c>
-      <c r="H8" s="25"/>
-      <c r="I8" s="25"/>
-    </row>
-    <row r="9" spans="1:9" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="21" t="s">
-        <v>138</v>
-      </c>
-      <c r="B9" s="23"/>
-      <c r="C9" s="23"/>
-      <c r="D9" s="23"/>
-      <c r="E9" s="25"/>
-      <c r="F9" s="25" t="s">
-        <v>139</v>
-      </c>
-      <c r="G9" s="25" t="s">
-        <v>139</v>
-      </c>
-      <c r="H9" s="25"/>
-      <c r="I9" s="25"/>
-    </row>
-    <row r="10" spans="1:9" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="21" t="s">
-        <v>140</v>
-      </c>
-      <c r="B10" s="23"/>
-      <c r="C10" s="23"/>
-      <c r="D10" s="23"/>
-      <c r="E10" s="25"/>
-      <c r="F10" s="25" t="s">
-        <v>139</v>
-      </c>
-      <c r="G10" s="25" t="s">
-        <v>139</v>
-      </c>
-      <c r="H10" s="25"/>
-      <c r="I10" s="25"/>
-    </row>
-    <row r="14" spans="1:9" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="27" t="s">
-        <v>141</v>
-      </c>
-      <c r="B14" s="22" t="s">
-        <v>142</v>
-      </c>
-      <c r="C14" s="26" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="21" t="s">
-        <v>144</v>
-      </c>
-      <c r="B15" s="23" t="s">
-        <v>145</v>
-      </c>
-      <c r="C15" s="23" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="21" t="s">
-        <v>147</v>
-      </c>
-      <c r="B16" s="23" t="s">
-        <v>148</v>
-      </c>
-      <c r="C16" s="23" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="21" t="s">
-        <v>119</v>
-      </c>
-      <c r="B17" s="23" t="s">
-        <v>150</v>
-      </c>
-      <c r="C17" s="23" t="s">
+      <c r="B21" s="22" t="s">
         <v>151</v>
+      </c>
+      <c r="C21" s="22" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="20" t="s">
+        <v>158</v>
+      </c>
+      <c r="B22" s="22"/>
+      <c r="C22" s="22"/>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A25" s="30" t="s">
+        <v>165</v>
+      </c>
+      <c r="B25" s="31" t="s">
+        <v>166</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B15" r:id="rId1" display="vscode-file://vscode-app/c:/Users/Ngoc/AppData/Local/Programs/Microsoft VS Code/1b50d58d73/resources/app/out/vs/code/electron-browser/workbench/workbench.html" xr:uid="{D0458559-2E72-4007-84AC-98B673B8E096}"/>
-    <hyperlink ref="B16" r:id="rId2" display="vscode-file://vscode-app/c:/Users/Ngoc/AppData/Local/Programs/Microsoft VS Code/1b50d58d73/resources/app/out/vs/code/electron-browser/workbench/workbench.html" xr:uid="{097AAD54-B361-4FCD-B84B-86C4490183F3}"/>
-    <hyperlink ref="B17" r:id="rId3" display="vscode-file://vscode-app/c:/Users/Ngoc/AppData/Local/Programs/Microsoft VS Code/1b50d58d73/resources/app/out/vs/code/electron-browser/workbench/workbench.html" xr:uid="{3FA5E5F5-2455-4168-989A-99F613E0E4E3}"/>
+    <hyperlink ref="B19" r:id="rId1" display="vscode-file://vscode-app/c:/Users/Ngoc/AppData/Local/Programs/Microsoft VS Code/1b50d58d73/resources/app/out/vs/code/electron-browser/workbench/workbench.html" xr:uid="{D0458559-2E72-4007-84AC-98B673B8E096}"/>
+    <hyperlink ref="B20" r:id="rId2" display="vscode-file://vscode-app/c:/Users/Ngoc/AppData/Local/Programs/Microsoft VS Code/1b50d58d73/resources/app/out/vs/code/electron-browser/workbench/workbench.html" xr:uid="{097AAD54-B361-4FCD-B84B-86C4490183F3}"/>
+    <hyperlink ref="B21" r:id="rId3" display="vscode-file://vscode-app/c:/Users/Ngoc/AppData/Local/Programs/Microsoft VS Code/1b50d58d73/resources/app/out/vs/code/electron-browser/workbench/workbench.html" xr:uid="{3FA5E5F5-2455-4168-989A-99F613E0E4E3}"/>
+    <hyperlink ref="A13" r:id="rId4" display="https://dashboard.ngrok.com/get-started/setup/windows" xr:uid="{83097FC5-91C2-4FB8-95FE-E4108F6691E3}"/>
+    <hyperlink ref="E13" r:id="rId5" xr:uid="{669C0AA8-1A60-494E-A0CE-9E3D5FA3E15F}"/>
+    <hyperlink ref="A25" r:id="rId6" display="https://sla-dashboard-9aoizetrr-mezyproject2026.vercel.app/" xr:uid="{844675C8-4108-427E-AE6D-0A7F8F045980}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId4"/>
+  <drawing r:id="rId7"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{41F0E622-BA0A-4026-9F4D-3E0A3D935EC8}">
+  <sheetPr codeName="Sheet4"/>
   <dimension ref="K1:L3"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="11:12" x14ac:dyDescent="0.25">
-      <c r="K1" s="28" t="s">
-        <v>152</v>
+      <c r="K1" s="27" t="s">
+        <v>153</v>
       </c>
     </row>
     <row r="2" spans="11:12" x14ac:dyDescent="0.25">
       <c r="L2" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
     </row>
     <row r="3" spans="11:12" x14ac:dyDescent="0.25">
       <c r="L3" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C0A8A570-8C52-4ACC-A500-1A8A87D624E4}">
+  <sheetPr codeName="Sheet5"/>
+  <dimension ref="K5:L23"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="11" max="11" width="29.25" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="5" spans="11:12" x14ac:dyDescent="0.25">
+      <c r="K5" s="28" t="s">
+        <v>156</v>
+      </c>
+      <c r="L5" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="20" spans="11:12" x14ac:dyDescent="0.25">
+      <c r="K20" t="s">
+        <v>163</v>
+      </c>
+      <c r="L20" s="28" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="23" spans="11:12" x14ac:dyDescent="0.25">
+      <c r="K23" s="28"/>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="K5" r:id="rId1" display="https://vercel.com/mezyproject2026/sla-dashboard/settings/domains?domainconnect-domain=sla.mezy.com.au" xr:uid="{045E6CD6-039B-4FB8-BFF3-AF6CFBEB03F1}"/>
+    <hyperlink ref="L20" r:id="rId2" display="https://vercel.com/mezyproject2026/sla-dashboard/deployments" xr:uid="{6E625930-FDFC-4DA8-8091-974BA2AE70DC}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A8A37160-CA21-47BC-9A50-A36042625CE1}">
+  <sheetPr codeName="Sheet6"/>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>